<commit_message>
Fix Estimated_Arrival to count ETA from pickup time
Time_taken in the historical data is measured from pickup, not order
time, so arrival was computed from the wrong start and could land
before the pickup. Arrival is now pickup + predicted ETA, rounded to the
nearest minute, with after-midnight pickups rolled to the next day.
Move the calculation to src/arrival.py, add tests, and regenerate
outputs. Predicted ETA and risk scores are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TRExKbT3kKXeBgU7NPXb7R
</commit_message>
<xml_diff>
--- a/outputs/active_deliveries_ZC_predicted.xlsx
+++ b/outputs/active_deliveries_ZC_predicted.xlsx
@@ -76,12 +76,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1881" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1881" uniqueCount="374">
   <si>
     <t xml:space="preserve">Active Deliveries (batch ZC): ETA and Risk Summary</t>
   </si>
   <si>
-    <t xml:space="preserve">Model run: 2026-09-26 05:04:15  |  Orders scored: 50</t>
+    <t xml:space="preserve">Model run: 2026-09-26 07:08:04  |  Orders scored: 50</t>
   </si>
   <si>
     <t xml:space="preserve">Risk category</t>
@@ -336,36 +336,36 @@
     <t xml:space="preserve">Weather: Windy</t>
   </si>
   <si>
+    <t xml:space="preserve">09:39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BANGRES12DEL02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09:05:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sunny</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buffet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">motorcycle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multiple deliveries: 1</t>
+  </si>
+  <si>
     <t xml:space="preserve">09:23</t>
   </si>
   <si>
-    <t xml:space="preserve">ZC-0002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BANGRES12DEL02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09:05:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sunny</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buffet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">motorcycle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multiple deliveries: 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09:18</t>
-  </si>
-  <si>
     <t xml:space="preserve">ZC-0003</t>
   </si>
   <si>
@@ -387,7 +387,7 @@
     <t xml:space="preserve">Weather: Stormy</t>
   </si>
   <si>
-    <t xml:space="preserve">09:13</t>
+    <t xml:space="preserve">09:28</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0004</t>
@@ -405,7 +405,7 @@
     <t xml:space="preserve">Weather: Windy; Multiple deliveries: 1</t>
   </si>
   <si>
-    <t xml:space="preserve">10:22</t>
+    <t xml:space="preserve">10:37</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0005</t>
@@ -423,7 +423,7 @@
     <t xml:space="preserve">Weather: Stormy; Multiple deliveries: 1</t>
   </si>
   <si>
-    <t xml:space="preserve">11:04</t>
+    <t xml:space="preserve">11:10</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0006</t>
@@ -438,7 +438,7 @@
     <t xml:space="preserve">11:05:00</t>
   </si>
   <si>
-    <t xml:space="preserve">11:15</t>
+    <t xml:space="preserve">11:30</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0007</t>
@@ -453,7 +453,7 @@
     <t xml:space="preserve">Weather: Sandstorms; Multiple deliveries: 1</t>
   </si>
   <si>
-    <t xml:space="preserve">11:13</t>
+    <t xml:space="preserve">11:29</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0008</t>
@@ -477,7 +477,7 @@
     <t xml:space="preserve">Weather: Sandstorms; Traffic: High; Multiple deliveries: 1</t>
   </si>
   <si>
-    <t xml:space="preserve">11:53</t>
+    <t xml:space="preserve">11:59</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0009</t>
@@ -498,7 +498,7 @@
     <t xml:space="preserve">Weather: Cloudy; Traffic: High</t>
   </si>
   <si>
-    <t xml:space="preserve">12:26</t>
+    <t xml:space="preserve">12:32</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0010</t>
@@ -519,7 +519,7 @@
     <t xml:space="preserve">Traffic: High; Multiple deliveries: 3</t>
   </si>
   <si>
-    <t xml:space="preserve">14:21</t>
+    <t xml:space="preserve">14:27</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0011</t>
@@ -537,7 +537,7 @@
     <t xml:space="preserve">Weather: Cloudy; Traffic: Medium; Multiple deliveries: 1</t>
   </si>
   <si>
-    <t xml:space="preserve">15:27</t>
+    <t xml:space="preserve">15:32</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0012</t>
@@ -555,7 +555,7 @@
     <t xml:space="preserve">Traffic: Medium; Multiple deliveries: 1</t>
   </si>
   <si>
-    <t xml:space="preserve">17:50</t>
+    <t xml:space="preserve">18:00</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0013</t>
@@ -573,7 +573,7 @@
     <t xml:space="preserve">Weather: Sandstorms; Traffic: Medium; Multiple deliveries: 1</t>
   </si>
   <si>
-    <t xml:space="preserve">17:58</t>
+    <t xml:space="preserve">18:03</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0014</t>
@@ -594,7 +594,7 @@
     <t xml:space="preserve">Weather: Fog; Traffic: Medium; Multiple deliveries: 1</t>
   </si>
   <si>
-    <t xml:space="preserve">17:57</t>
+    <t xml:space="preserve">18:08</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0015</t>
@@ -609,7 +609,7 @@
     <t xml:space="preserve">Weather: Windy; Traffic: Medium; Multiple deliveries: 1</t>
   </si>
   <si>
-    <t xml:space="preserve">18:14</t>
+    <t xml:space="preserve">18:30</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0016</t>
@@ -621,7 +621,7 @@
     <t xml:space="preserve">18:00:00</t>
   </si>
   <si>
-    <t xml:space="preserve">18:06</t>
+    <t xml:space="preserve">18:16</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0017</t>
@@ -639,7 +639,7 @@
     <t xml:space="preserve">Traffic: Medium</t>
   </si>
   <si>
-    <t xml:space="preserve">18:48</t>
+    <t xml:space="preserve">19:03</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0018</t>
@@ -654,7 +654,7 @@
     <t xml:space="preserve">18:35:00</t>
   </si>
   <si>
-    <t xml:space="preserve">18:41</t>
+    <t xml:space="preserve">18:57</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0019</t>
@@ -666,7 +666,7 @@
     <t xml:space="preserve">Weather: Cloudy; Traffic: Medium</t>
   </si>
   <si>
-    <t xml:space="preserve">18:37</t>
+    <t xml:space="preserve">18:52</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0020</t>
@@ -681,7 +681,7 @@
     <t xml:space="preserve">18:40:00</t>
   </si>
   <si>
-    <t xml:space="preserve">18:44</t>
+    <t xml:space="preserve">18:54</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0021</t>
@@ -693,7 +693,7 @@
     <t xml:space="preserve">18:45:00</t>
   </si>
   <si>
-    <t xml:space="preserve">18:59</t>
+    <t xml:space="preserve">19:04</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0022</t>
@@ -705,7 +705,7 @@
     <t xml:space="preserve">18:55:00</t>
   </si>
   <si>
-    <t xml:space="preserve">19:05</t>
+    <t xml:space="preserve">19:16</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0023</t>
@@ -732,7 +732,7 @@
     <t xml:space="preserve">00:15:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:14</t>
+    <t xml:space="preserve">00:30</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0025</t>
@@ -747,339 +747,342 @@
     <t xml:space="preserve">Weather: Cloudy; Multiple deliveries: 1</t>
   </si>
   <si>
+    <t xml:space="preserve">00:25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHENRES19DEL03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:10:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:20:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Severe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather: Cloudy; Traffic: Jam; Multiple deliveries: 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COIMBRES03DEL02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:15:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:30:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather: Windy; Traffic: Jam; Multiple deliveries: 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AGRRES04DEL02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:25:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traffic: Jam; Multiple deliveries: 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RANCHIRES18DEL01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:55:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather: Sandstorms; Traffic: Jam; Multiple deliveries: 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COIMBRES01DEL02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:15:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather: Windy; Traffic: Jam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0031</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RANCHIRES08DEL01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather: Fog; Traffic: Jam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:56</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SURRES03DEL03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:20:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:35:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather: Sandstorms; Traffic: Jam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0033</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MYSRES13DEL01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:40:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather: Stormy; Traffic: Jam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KOLRES12DEL01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:45:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather: Stormy; Traffic: Jam; Multiple deliveries: 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0036</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KOLRES17DEL03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:55:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JAPRES09DEL03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:05:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MUMRES05DEL02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:15:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:30:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:25:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:35:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22:12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VADRES20DEL01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:40:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather: Fog; Traffic: Jam; Multiple deliveries: 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COIMBRES19DEL03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:50:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22:17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BANGRES17DEL03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22:10:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22:15:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22:38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BANGRES19DEL02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22:40:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22:55:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23:14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHENRES18DEL03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22:50:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23:05:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23:21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LUDHRES11DEL01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23:37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BANGRES010DEL02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHENRES12DEL01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather: Fog; Multiple deliveries: 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23:45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZC-0048</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SURRES01DEL02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23:35:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23:50:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">00:15</t>
   </si>
   <si>
-    <t xml:space="preserve">ZC-0026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHENRES19DEL03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:10:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:20:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Severe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather: Cloudy; Traffic: Jam; Multiple deliveries: 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COIMBRES03DEL02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:15:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:30:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather: Windy; Traffic: Jam; Multiple deliveries: 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:34</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0028</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AGRRES04DEL02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:25:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Traffic: Jam; Multiple deliveries: 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0029</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RANCHIRES18DEL01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:55:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather: Sandstorms; Traffic: Jam; Multiple deliveries: 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COIMBRES01DEL02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:15:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather: Windy; Traffic: Jam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0031</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RANCHIRES08DEL01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather: Fog; Traffic: Jam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0032</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SURRES03DEL03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:20:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:35:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather: Sandstorms; Traffic: Jam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:57</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0033</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MYSRES13DEL01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:40:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather: Stormy; Traffic: Jam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:55</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0034</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KOLRES12DEL01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:45:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather: Stormy; Traffic: Jam; Multiple deliveries: 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0035</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0036</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KOLRES17DEL03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:55:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0037</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JAPRES09DEL03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:05:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0038</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MUMRES05DEL02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:15:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:30:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:44</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0039</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:25:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:35:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22:02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0040</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VADRES20DEL01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:40:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather: Fog; Traffic: Jam; Multiple deliveries: 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22:14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0041</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COIMBRES19DEL03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:50:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22:06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0042</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BANGRES17DEL03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22:10:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22:15:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22:33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0043</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BANGRES19DEL02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22:40:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22:55:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22:58</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0044</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHENRES18DEL03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22:50:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23:05:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23:05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0045</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LUDHRES11DEL01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23:31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0046</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BANGRES010DEL02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23:09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0047</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHENRES12DEL01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather: Fog; Multiple deliveries: 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZC-0048</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SURRES01DEL02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23:35:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23:50:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23:59</t>
-  </si>
-  <si>
     <t xml:space="preserve">ZC-0049</t>
   </si>
   <si>
@@ -1092,7 +1095,7 @@
     <t xml:space="preserve">23:55:00</t>
   </si>
   <si>
-    <t xml:space="preserve">23:54</t>
+    <t xml:space="preserve">00:10</t>
   </si>
   <si>
     <t xml:space="preserve">ZC-0050</t>
@@ -1101,7 +1104,7 @@
     <t xml:space="preserve">SURRES010DEL02</t>
   </si>
   <si>
-    <t xml:space="preserve">00:11</t>
+    <t xml:space="preserve">00:26</t>
   </si>
   <si>
     <t xml:space="preserve">Risk scoring rules (edit blue cells; Active_Deliveries recalculates)</t>
@@ -2403,7 +2406,7 @@
         <v>23.8</v>
       </c>
       <c r="V2" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W2" s="20" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE2+AF2+AG2+AH2)</f>
@@ -2516,7 +2519,7 @@
         <v>18.2</v>
       </c>
       <c r="V3" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W3" s="20" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE3+AF3+AG3+AH3)</f>
@@ -2629,7 +2632,7 @@
         <v>13.4</v>
       </c>
       <c r="V4" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W4" s="20" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE4+AF4+AG4+AH4)</f>
@@ -2742,7 +2745,7 @@
         <v>22.1</v>
       </c>
       <c r="V5" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W5" s="20" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE5+AF5+AG5+AH5)</f>
@@ -2855,7 +2858,7 @@
         <v>24.6</v>
       </c>
       <c r="V6" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W6" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE6+AF6+AG6+AH6)</f>
@@ -2968,7 +2971,7 @@
         <v>25.1</v>
       </c>
       <c r="V7" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W7" s="20" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE7+AF7+AG7+AH7)</f>
@@ -3081,7 +3084,7 @@
         <v>23.8</v>
       </c>
       <c r="V8" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W8" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE8+AF8+AG8+AH8)</f>
@@ -3194,7 +3197,7 @@
         <v>28.6</v>
       </c>
       <c r="V9" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W9" s="22" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE9+AF9+AG9+AH9)</f>
@@ -3307,7 +3310,7 @@
         <v>26.7</v>
       </c>
       <c r="V10" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W10" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE10+AF10+AG10+AH10)</f>
@@ -3420,7 +3423,7 @@
         <v>51.8</v>
       </c>
       <c r="V11" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W11" s="22" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE11+AF11+AG11+AH11)</f>
@@ -3533,7 +3536,7 @@
         <v>17.4</v>
       </c>
       <c r="V12" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W12" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE12+AF12+AG12+AH12)</f>
@@ -3646,7 +3649,7 @@
         <v>30.4</v>
       </c>
       <c r="V13" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W13" s="20" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE13+AF13+AG13+AH13)</f>
@@ -3759,7 +3762,7 @@
         <v>23</v>
       </c>
       <c r="V14" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W14" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE14+AF14+AG14+AH14)</f>
@@ -3872,7 +3875,7 @@
         <v>17.7</v>
       </c>
       <c r="V15" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W15" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE15+AF15+AG15+AH15)</f>
@@ -3985,7 +3988,7 @@
         <v>34.6</v>
       </c>
       <c r="V16" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W16" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE16+AF16+AG16+AH16)</f>
@@ -4098,7 +4101,7 @@
         <v>16.5</v>
       </c>
       <c r="V17" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W17" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE17+AF17+AG17+AH17)</f>
@@ -4211,7 +4214,7 @@
         <v>38.2</v>
       </c>
       <c r="V18" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W18" s="20" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE18+AF18+AG18+AH18)</f>
@@ -4324,7 +4327,7 @@
         <v>21.6</v>
       </c>
       <c r="V19" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W19" s="20" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE19+AF19+AG19+AH19)</f>
@@ -4437,7 +4440,7 @@
         <v>17.2</v>
       </c>
       <c r="V20" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W20" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE20+AF20+AG20+AH20)</f>
@@ -4550,7 +4553,7 @@
         <v>14.3</v>
       </c>
       <c r="V21" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W21" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE21+AF21+AG21+AH21)</f>
@@ -4663,7 +4666,7 @@
         <v>19.5</v>
       </c>
       <c r="V22" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W22" s="20" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE22+AF22+AG22+AH22)</f>
@@ -4776,7 +4779,7 @@
         <v>20.9</v>
       </c>
       <c r="V23" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W23" s="20" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE23+AF23+AG23+AH23)</f>
@@ -4889,7 +4892,7 @@
         <v>14.3</v>
       </c>
       <c r="V24" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W24" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE24+AF24+AG24+AH24)</f>
@@ -5002,7 +5005,7 @@
         <v>14.9</v>
       </c>
       <c r="V25" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W25" s="20" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE25+AF25+AG25+AH25)</f>
@@ -5115,7 +5118,7 @@
         <v>15</v>
       </c>
       <c r="V26" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W26" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE26+AF26+AG26+AH26)</f>
@@ -5228,7 +5231,7 @@
         <v>35.4</v>
       </c>
       <c r="V27" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W27" s="22" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE27+AF27+AG27+AH27)</f>
@@ -5341,7 +5344,7 @@
         <v>19.1</v>
       </c>
       <c r="V28" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W28" s="22" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE28+AF28+AG28+AH28)</f>
@@ -5454,7 +5457,7 @@
         <v>18.5</v>
       </c>
       <c r="V29" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W29" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE29+AF29+AG29+AH29)</f>
@@ -5567,7 +5570,7 @@
         <v>32.5</v>
       </c>
       <c r="V30" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W30" s="22" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE30+AF30+AG30+AH30)</f>
@@ -5680,7 +5683,7 @@
         <v>21.6</v>
       </c>
       <c r="V31" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W31" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE31+AF31+AG31+AH31)</f>
@@ -5793,7 +5796,7 @@
         <v>40.8</v>
       </c>
       <c r="V32" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W32" s="22" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE32+AF32+AG32+AH32)</f>
@@ -5906,7 +5909,7 @@
         <v>37.6</v>
       </c>
       <c r="V33" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W33" s="22" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE33+AF33+AG33+AH33)</f>
@@ -6019,7 +6022,7 @@
         <v>20.8</v>
       </c>
       <c r="V34" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W34" s="22" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE34+AF34+AG34+AH34)</f>
@@ -6132,7 +6135,7 @@
         <v>22.8</v>
       </c>
       <c r="V35" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W35" s="22" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE35+AF35+AG35+AH35)</f>
@@ -6245,7 +6248,7 @@
         <v>36.8</v>
       </c>
       <c r="V36" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W36" s="22" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE36+AF36+AG36+AH36)</f>
@@ -6358,7 +6361,7 @@
         <v>27.8</v>
       </c>
       <c r="V37" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W37" s="22" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE37+AF37+AG37+AH37)</f>
@@ -6471,7 +6474,7 @@
         <v>22.4</v>
       </c>
       <c r="V38" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W38" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE38+AF38+AG38+AH38)</f>
@@ -6516,15 +6519,15 @@
         <v>13.41</v>
       </c>
       <c r="AK38" s="18" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="18" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B39" s="18" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C39" s="18" t="n">
         <v>30</v>
@@ -6548,10 +6551,10 @@
         <v>73</v>
       </c>
       <c r="J39" s="18" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="K39" s="18" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="L39" s="18" t="s">
         <v>90</v>
@@ -6584,7 +6587,7 @@
         <v>29.8</v>
       </c>
       <c r="V39" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W39" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE39+AF39+AG39+AH39)</f>
@@ -6629,12 +6632,12 @@
         <v>12.24</v>
       </c>
       <c r="AK39" s="18" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="18" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B40" s="18" t="s">
         <v>111</v>
@@ -6661,10 +6664,10 @@
         <v>73</v>
       </c>
       <c r="J40" s="18" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="K40" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L40" s="18" t="s">
         <v>76</v>
@@ -6697,7 +6700,7 @@
         <v>37</v>
       </c>
       <c r="V40" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W40" s="22" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE40+AF40+AG40+AH40)</f>
@@ -6742,15 +6745,15 @@
         <v>7.77</v>
       </c>
       <c r="AK40" s="18" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="18" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B41" s="18" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C41" s="18" t="n">
         <v>38</v>
@@ -6774,10 +6777,10 @@
         <v>73</v>
       </c>
       <c r="J41" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K41" s="18" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L41" s="18" t="s">
         <v>169</v>
@@ -6810,7 +6813,7 @@
         <v>39.7</v>
       </c>
       <c r="V41" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W41" s="22" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE41+AF41+AG41+AH41)</f>
@@ -6849,21 +6852,21 @@
         <v>10</v>
       </c>
       <c r="AI41" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="AJ41" s="18" t="n">
         <v>10.6</v>
       </c>
       <c r="AK41" s="18" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="18" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B42" s="18" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C42" s="18" t="n">
         <v>24</v>
@@ -6887,10 +6890,10 @@
         <v>73</v>
       </c>
       <c r="J42" s="18" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="K42" s="18" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L42" s="18" t="s">
         <v>169</v>
@@ -6923,7 +6926,7 @@
         <v>26.9</v>
       </c>
       <c r="V42" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W42" s="22" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE42+AF42+AG42+AH42)</f>
@@ -6962,21 +6965,21 @@
         <v>10</v>
       </c>
       <c r="AI42" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="AJ42" s="18" t="n">
         <v>4.67</v>
       </c>
       <c r="AK42" s="18" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="18" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B43" s="18" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C43" s="18" t="n">
         <v>30</v>
@@ -7000,10 +7003,10 @@
         <v>73</v>
       </c>
       <c r="J43" s="18" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="K43" s="18" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="L43" s="18" t="s">
         <v>123</v>
@@ -7036,7 +7039,7 @@
         <v>23.2</v>
       </c>
       <c r="V43" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W43" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE43+AF43+AG43+AH43)</f>
@@ -7081,15 +7084,15 @@
         <v>13.97</v>
       </c>
       <c r="AK43" s="18" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="18" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B44" s="18" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C44" s="18" t="n">
         <v>21</v>
@@ -7113,10 +7116,10 @@
         <v>73</v>
       </c>
       <c r="J44" s="18" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="K44" s="18" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="L44" s="18" t="s">
         <v>90</v>
@@ -7149,7 +7152,7 @@
         <v>18.5</v>
       </c>
       <c r="V44" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W44" s="20" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE44+AF44+AG44+AH44)</f>
@@ -7188,21 +7191,21 @@
         <v>0</v>
       </c>
       <c r="AI44" s="18" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="AJ44" s="18" t="n">
         <v>7.76</v>
       </c>
       <c r="AK44" s="18" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="18" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B45" s="18" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C45" s="18" t="n">
         <v>27</v>
@@ -7226,10 +7229,10 @@
         <v>73</v>
       </c>
       <c r="J45" s="18" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="K45" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="L45" s="18" t="s">
         <v>123</v>
@@ -7262,7 +7265,7 @@
         <v>15.7</v>
       </c>
       <c r="V45" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W45" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE45+AF45+AG45+AH45)</f>
@@ -7307,15 +7310,15 @@
         <v>13.97</v>
       </c>
       <c r="AK45" s="18" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="18" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B46" s="18" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C46" s="18" t="n">
         <v>31</v>
@@ -7339,10 +7342,10 @@
         <v>73</v>
       </c>
       <c r="J46" s="18" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="K46" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="L46" s="18" t="s">
         <v>138</v>
@@ -7375,7 +7378,7 @@
         <v>36.8</v>
       </c>
       <c r="V46" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W46" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE46+AF46+AG46+AH46)</f>
@@ -7420,15 +7423,15 @@
         <v>16.11</v>
       </c>
       <c r="AK46" s="18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="18" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B47" s="18" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C47" s="18" t="n">
         <v>22</v>
@@ -7452,10 +7455,10 @@
         <v>73</v>
       </c>
       <c r="J47" s="18" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="K47" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="L47" s="18" t="s">
         <v>98</v>
@@ -7488,7 +7491,7 @@
         <v>14.5</v>
       </c>
       <c r="V47" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W47" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE47+AF47+AG47+AH47)</f>
@@ -7533,15 +7536,15 @@
         <v>20.18</v>
       </c>
       <c r="AK47" s="18" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B48" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C48" s="18" t="n">
         <v>35</v>
@@ -7565,10 +7568,10 @@
         <v>73</v>
       </c>
       <c r="J48" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="K48" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="L48" s="18" t="s">
         <v>169</v>
@@ -7601,7 +7604,7 @@
         <v>40</v>
       </c>
       <c r="V48" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W48" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE48+AF48+AG48+AH48)</f>
@@ -7640,21 +7643,21 @@
         <v>20</v>
       </c>
       <c r="AI48" s="18" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="AJ48" s="18" t="n">
         <v>10.87</v>
       </c>
       <c r="AK48" s="18" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="18" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B49" s="18" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C49" s="18" t="n">
         <v>32</v>
@@ -7678,10 +7681,10 @@
         <v>73</v>
       </c>
       <c r="J49" s="18" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="K49" s="18" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="L49" s="18" t="s">
         <v>76</v>
@@ -7714,7 +7717,7 @@
         <v>24.6</v>
       </c>
       <c r="V49" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W49" s="20" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE49+AF49+AG49+AH49)</f>
@@ -7759,15 +7762,15 @@
         <v>19.76</v>
       </c>
       <c r="AK49" s="18" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="18" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B50" s="18" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C50" s="18" t="n">
         <v>21</v>
@@ -7791,10 +7794,10 @@
         <v>73</v>
       </c>
       <c r="J50" s="18" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="K50" s="18" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="L50" s="18" t="s">
         <v>76</v>
@@ -7827,7 +7830,7 @@
         <v>14.5</v>
       </c>
       <c r="V50" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W50" s="20" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE50+AF50+AG50+AH50)</f>
@@ -7872,15 +7875,15 @@
         <v>13.63</v>
       </c>
       <c r="AK50" s="18" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="18" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B51" s="18" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C51" s="18" t="n">
         <v>27</v>
@@ -7904,7 +7907,7 @@
         <v>73</v>
       </c>
       <c r="J51" s="18" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="K51" s="18" t="s">
         <v>221</v>
@@ -7940,7 +7943,7 @@
         <v>16.1</v>
       </c>
       <c r="V51" s="19" t="n">
-        <v>46291.2112847222</v>
+        <v>46291.2972685185</v>
       </c>
       <c r="W51" s="21" t="n">
         <f aca="false">MIN(Risk_Rules!$B$27,AE51+AF51+AG51+AH51)</f>
@@ -7985,7 +7988,7 @@
         <v>7.6</v>
       </c>
       <c r="AK51" s="18" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
   </sheetData>
@@ -8017,28 +8020,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="23" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="24" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8109,18 +8112,18 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="24" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B14" s="24" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8169,18 +8172,18 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="24" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B21" s="24" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C21" s="24" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8196,23 +8199,23 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B23" s="25" t="n">
         <v>30</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B26" s="25" t="n">
         <v>10</v>
@@ -8220,7 +8223,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B27" s="25" t="n">
         <v>100</v>
@@ -8228,18 +8231,18 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B30" s="24" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C30" s="24" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8250,7 +8253,7 @@
         <v>70</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8261,7 +8264,7 @@
         <v>50</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8272,7 +8275,7 @@
         <v>30</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8283,7 +8286,7 @@
         <v>0</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
   </sheetData>
@@ -8327,7 +8330,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8391,19 +8394,19 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C4" s="18" t="s">
         <v>80</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F4" s="18" t="s">
         <v>169</v>
@@ -8436,7 +8439,7 @@
         <v>39.7</v>
       </c>
       <c r="P4" s="18" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="Q4" s="22" t="n">
         <v>60</v>
@@ -8445,7 +8448,7 @@
         <v>8</v>
       </c>
       <c r="S4" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8686,19 +8689,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C9" s="18" t="s">
         <v>80</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F9" s="18" t="s">
         <v>169</v>
@@ -8731,7 +8734,7 @@
         <v>26.9</v>
       </c>
       <c r="P9" s="18" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="Q9" s="22" t="n">
         <v>60</v>
@@ -8740,7 +8743,7 @@
         <v>8</v>
       </c>
       <c r="S9" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8981,7 +8984,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B14" s="18" t="s">
         <v>111</v>
@@ -8990,10 +8993,10 @@
         <v>80</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F14" s="18" t="s">
         <v>76</v>
@@ -9026,7 +9029,7 @@
         <v>37</v>
       </c>
       <c r="P14" s="18" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="Q14" s="22" t="n">
         <v>50</v>
@@ -9258,7 +9261,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9322,19 +9325,19 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C4" s="18" t="s">
         <v>80</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F4" s="18" t="s">
         <v>169</v>
@@ -9367,7 +9370,7 @@
         <v>40</v>
       </c>
       <c r="P4" s="18" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="Q4" s="21" t="n">
         <v>40</v>
@@ -9376,24 +9379,24 @@
         <v>9</v>
       </c>
       <c r="S4" s="18" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C5" s="18" t="s">
         <v>80</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F5" s="18" t="s">
         <v>90</v>
@@ -9426,7 +9429,7 @@
         <v>29.8</v>
       </c>
       <c r="P5" s="18" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="Q5" s="21" t="n">
         <v>40</v>
@@ -9603,7 +9606,7 @@
         <v>22.4</v>
       </c>
       <c r="P8" s="18" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="Q8" s="21" t="n">
         <v>40</v>
@@ -9971,19 +9974,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C15" s="18" t="s">
         <v>100</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F15" s="18" t="s">
         <v>138</v>
@@ -10016,7 +10019,7 @@
         <v>36.8</v>
       </c>
       <c r="P15" s="18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="Q15" s="21" t="n">
         <v>30</v>
@@ -10207,19 +10210,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C19" s="18" t="s">
         <v>80</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F19" s="18" t="s">
         <v>123</v>
@@ -10252,7 +10255,7 @@
         <v>23.2</v>
       </c>
       <c r="P19" s="18" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Q19" s="21" t="n">
         <v>30</v>
@@ -10325,16 +10328,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C21" s="18" t="s">
         <v>80</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E21" s="18" t="s">
         <v>221</v>
@@ -10370,7 +10373,7 @@
         <v>16.1</v>
       </c>
       <c r="P21" s="18" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="Q21" s="21" t="n">
         <v>30</v>
@@ -10384,19 +10387,19 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C22" s="18" t="s">
         <v>100</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F22" s="18" t="s">
         <v>123</v>
@@ -10429,7 +10432,7 @@
         <v>15.7</v>
       </c>
       <c r="P22" s="18" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="Q22" s="21" t="n">
         <v>30</v>
@@ -10502,19 +10505,19 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C24" s="18" t="s">
         <v>100</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F24" s="18" t="s">
         <v>98</v>
@@ -10547,7 +10550,7 @@
         <v>14.5</v>
       </c>
       <c r="P24" s="18" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="Q24" s="21" t="n">
         <v>30</v>
@@ -10856,19 +10859,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="18" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C30" s="18" t="s">
         <v>100</v>
       </c>
       <c r="D30" s="18" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F30" s="18" t="s">
         <v>76</v>
@@ -10901,7 +10904,7 @@
         <v>14.5</v>
       </c>
       <c r="P30" s="18" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="Q30" s="20" t="n">
         <v>20</v>
@@ -11033,19 +11036,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="18" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C33" s="18" t="s">
         <v>80</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E33" s="18" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F33" s="18" t="s">
         <v>76</v>
@@ -11078,7 +11081,7 @@
         <v>24.6</v>
       </c>
       <c r="P33" s="18" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="Q33" s="20" t="n">
         <v>10</v>
@@ -11387,19 +11390,19 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="18" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B39" s="18" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C39" s="18" t="s">
         <v>80</v>
       </c>
       <c r="D39" s="18" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E39" s="18" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F39" s="18" t="s">
         <v>90</v>
@@ -11432,16 +11435,16 @@
         <v>18.5</v>
       </c>
       <c r="P39" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="Q39" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="S39" s="18" t="s">
         <v>312</v>
-      </c>
-      <c r="Q39" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="R39" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="S39" s="18" t="s">
-        <v>311</v>
       </c>
     </row>
   </sheetData>
@@ -11478,7 +11481,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11492,16 +11495,16 @@
         <v>54</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="I3" s="15" t="n">
         <f aca="false">AVERAGE(F4:F53)</f>
@@ -11530,7 +11533,7 @@
         <v>0.800000000000001</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="I4" s="15" t="n">
         <f aca="false">SQRT(SUMPRODUCT(E4:E53,E4:E53)/COUNT(E4:E53))</f>
@@ -11559,7 +11562,7 @@
         <v>2.2</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="I5" s="15" t="n">
         <f aca="false">AVERAGE(E4:E53)</f>
@@ -11588,7 +11591,7 @@
         <v>1.4</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="I6" s="6" t="n">
         <f aca="false">COUNTIF(F4:F53,"&lt;=5")/COUNT(F4:F53)</f>
@@ -12345,7 +12348,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>9</v>
@@ -12367,7 +12370,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>8</v>
@@ -12389,7 +12392,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>8</v>
@@ -12411,7 +12414,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B44" s="5" t="s">
         <v>8</v>
@@ -12433,7 +12436,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>9</v>
@@ -12455,7 +12458,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B46" s="5" t="s">
         <v>10</v>
@@ -12477,7 +12480,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>9</v>
@@ -12499,7 +12502,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>9</v>
@@ -12521,7 +12524,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>9</v>
@@ -12543,7 +12546,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>9</v>
@@ -12565,7 +12568,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>10</v>
@@ -12587,7 +12590,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>10</v>
@@ -12609,7 +12612,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>9</v>

</xml_diff>